<commit_message>
fix(spec): round panel area to match Excel calculation
The area per panel is now rounded to 3 decimal places before summation to ensure the total area matches manual Excel calculations. This prevents floating-point precision discrepancies in the final specification output.
</commit_message>
<xml_diff>
--- a/Для разработчиков ИИ (extract.me)/Склад_раслкдка панелей_23.04.2026_spec.xlsx
+++ b/Для разработчиков ИИ (extract.me)/Склад_раслкдка панелей_23.04.2026_spec.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Панели" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Панели" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -856,7 +856,7 @@
         <v>8</v>
       </c>
       <c r="P8" t="n">
-        <v>14.185</v>
+        <v>14.184</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -984,7 +984,7 @@
         <v>5</v>
       </c>
       <c r="P10" t="n">
-        <v>21.956</v>
+        <v>21.955</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
         <v>7</v>
       </c>
       <c r="P11" t="n">
-        <v>48.231</v>
+        <v>48.23</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
         <v>112</v>
       </c>
       <c r="P12" t="n">
-        <v>797.014</v>
+        <v>796.992</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1176,7 +1176,7 @@
         <v>16</v>
       </c>
       <c r="P13" t="n">
-        <v>117.477</v>
+        <v>117.472</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1240,7 +1240,7 @@
         <v>8</v>
       </c>
       <c r="P14" t="n">
-        <v>60.357</v>
+        <v>60.36</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
         <v>420</v>
       </c>
       <c r="M15" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N15" t="n">
         <v>150</v>
@@ -1304,7 +1304,7 @@
         <v>1</v>
       </c>
       <c r="P15" t="n">
-        <v>0.42</v>
+        <v>0.5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1359,7 +1359,7 @@
         <v>430</v>
       </c>
       <c r="M16" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N16" t="n">
         <v>150</v>
@@ -1368,7 +1368,7 @@
         <v>1</v>
       </c>
       <c r="P16" t="n">
-        <v>0.43</v>
+        <v>0.512</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
         <v>570</v>
       </c>
       <c r="M17" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N17" t="n">
         <v>150</v>
@@ -1432,7 +1432,7 @@
         <v>2</v>
       </c>
       <c r="P17" t="n">
-        <v>1.14</v>
+        <v>1.356</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
         <v>1400</v>
       </c>
       <c r="M18" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N18" t="n">
         <v>150</v>
@@ -1496,7 +1496,7 @@
         <v>2</v>
       </c>
       <c r="P18" t="n">
-        <v>2.8</v>
+        <v>3.332</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -1551,7 +1551,7 @@
         <v>1990</v>
       </c>
       <c r="M19" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N19" t="n">
         <v>150</v>
@@ -1560,7 +1560,7 @@
         <v>56</v>
       </c>
       <c r="P19" t="n">
-        <v>111.44</v>
+        <v>132.608</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         <v>2180</v>
       </c>
       <c r="M20" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N20" t="n">
         <v>150</v>
@@ -1624,7 +1624,7 @@
         <v>1</v>
       </c>
       <c r="P20" t="n">
-        <v>2.18</v>
+        <v>2.594</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
         <v>2350</v>
       </c>
       <c r="M21" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N21" t="n">
         <v>150</v>
@@ -1688,7 +1688,7 @@
         <v>1</v>
       </c>
       <c r="P21" t="n">
-        <v>2.35</v>
+        <v>2.796</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -1743,7 +1743,7 @@
         <v>2390</v>
       </c>
       <c r="M22" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N22" t="n">
         <v>150</v>
@@ -1752,7 +1752,7 @@
         <v>4</v>
       </c>
       <c r="P22" t="n">
-        <v>9.56</v>
+        <v>11.376</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
         <v>2540</v>
       </c>
       <c r="M23" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N23" t="n">
         <v>150</v>
@@ -1816,7 +1816,7 @@
         <v>1</v>
       </c>
       <c r="P23" t="n">
-        <v>2.54</v>
+        <v>3.023</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
         <v>4090</v>
       </c>
       <c r="M24" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N24" t="n">
         <v>150</v>
@@ -1880,7 +1880,7 @@
         <v>4</v>
       </c>
       <c r="P24" t="n">
-        <v>16.36</v>
+        <v>19.468</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -1935,7 +1935,7 @@
         <v>4540</v>
       </c>
       <c r="M25" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N25" t="n">
         <v>150</v>
@@ -1944,7 +1944,7 @@
         <v>1</v>
       </c>
       <c r="P25" t="n">
-        <v>4.54</v>
+        <v>5.403</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -1999,7 +1999,7 @@
         <v>4560</v>
       </c>
       <c r="M26" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N26" t="n">
         <v>150</v>
@@ -2008,7 +2008,7 @@
         <v>2</v>
       </c>
       <c r="P26" t="n">
-        <v>9.119999999999999</v>
+        <v>10.852</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2063,7 +2063,7 @@
         <v>5620</v>
       </c>
       <c r="M27" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N27" t="n">
         <v>150</v>
@@ -2072,7 +2072,7 @@
         <v>9</v>
       </c>
       <c r="P27" t="n">
-        <v>50.58</v>
+        <v>60.192</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
         <v>5980</v>
       </c>
       <c r="M28" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N28" t="n">
         <v>150</v>
@@ -2136,7 +2136,7 @@
         <v>451</v>
       </c>
       <c r="P28" t="n">
-        <v>2696.98</v>
+        <v>3209.316</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -2191,7 +2191,7 @@
         <v>6170</v>
       </c>
       <c r="M29" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N29" t="n">
         <v>150</v>
@@ -2200,7 +2200,7 @@
         <v>25</v>
       </c>
       <c r="P29" t="n">
-        <v>154.25</v>
+        <v>183.55</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -2255,7 +2255,7 @@
         <v>6340</v>
       </c>
       <c r="M30" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N30" t="n">
         <v>150</v>
@@ -2264,7 +2264,7 @@
         <v>33</v>
       </c>
       <c r="P30" t="n">
-        <v>209.22</v>
+        <v>248.985</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -2319,7 +2319,7 @@
         <v>6820</v>
       </c>
       <c r="M31" t="n">
-        <v>1000</v>
+        <v>1190</v>
       </c>
       <c r="N31" t="n">
         <v>150</v>
@@ -2328,7 +2328,7 @@
         <v>1</v>
       </c>
       <c r="P31" t="n">
-        <v>6.82</v>
+        <v>8.116</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         <v>784</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>4444.92</v>
+        <v>5068.142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>